<commit_message>
conteo 26/09 corregido con Coronel Raiz (cam 2 y 5 son Brasil): BR 11653, PY 13673, BO 1646; + carpetas de importacion 2026 pegadas por Gonzalo (tsv)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fuentes/stock/2026-09-26_conteo_camaras.xlsx
+++ b/fuentes/stock/2026-09-26_conteo_camaras.xlsx
@@ -9,13 +9,14 @@
     <sheet name="ecuador_zac" sheetId="2" r:id="rId3"/>
     <sheet name="bolivia" sheetId="3" r:id="rId4"/>
     <sheet name="zac_erp_por_camara" sheetId="4" r:id="rId5"/>
+    <sheet name="cr_erp_por_camara" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="91">
   <si>
     <t>fecha</t>
   </si>
@@ -269,10 +270,25 @@
     <t>Coronel Raiz</t>
   </si>
   <si>
-    <t>Banana Paraguay Pepe (supuesto)</t>
-  </si>
-  <si>
-    <t>Brasil (supuesto)</t>
+    <t>(vacia)</t>
+  </si>
+  <si>
+    <t>Palta</t>
+  </si>
+  <si>
+    <t>Pina</t>
+  </si>
+  <si>
+    <t>Jengibre</t>
+  </si>
+  <si>
+    <t>Platano</t>
+  </si>
+  <si>
+    <t>Melon Cantalupe</t>
+  </si>
+  <si>
+    <t>Sandia</t>
   </si>
 </sst>
 </file>
@@ -1121,7 +1137,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11.829548835754395" customWidth="1"/>
@@ -1912,44 +1928,342 @@
         <v>750</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="B40" s="0" t="s">
+  </sheetData>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="11.829548835754395" customWidth="1"/>
+    <col min="2" max="2" width="12.3339204788208" customWidth="1"/>
+    <col min="3" max="3" width="10.814667701721191" customWidth="1"/>
+    <col min="4" max="4" width="20.482635498046875" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" customWidth="1"/>
+    <col min="6" max="6" width="9.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="0" t="s">
         <v>83</v>
       </c>
-      <c r="C40" s="0" t="s">
+      <c r="C2" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2" s="0">
+        <v>3024</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="C3" s="0" t="s">
         <v>47</v>
       </c>
-      <c r="D40" s="0" t="s">
+      <c r="D3" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="F3" s="0">
+        <v>1944</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="0">
+        <v>1080</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>54</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="E5" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="F5" s="0">
+        <v>2160</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="E6" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6" s="0">
+        <v>1080</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="D7" s="0" t="s">
         <v>84</v>
       </c>
-      <c r="E40" s="0" t="s">
-        <v>51</v>
-      </c>
-      <c r="F40" s="0">
-        <v>1944</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="B41" s="0" t="s">
+      <c r="E7" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="s">
         <v>83</v>
       </c>
-      <c r="C41" s="0" t="s">
+      <c r="C8" s="0" t="s">
         <v>56</v>
       </c>
-      <c r="D41" s="0" t="s">
+      <c r="D8" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="E8" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="F8" s="0">
+        <v>1080</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="C9" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="D9" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="E9" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="F9" s="0">
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="C10" s="0" t="s">
+        <v>57</v>
+      </c>
+      <c r="D10" s="0" t="s">
         <v>85</v>
       </c>
-      <c r="E41" s="0" t="s">
-        <v>49</v>
-      </c>
-      <c r="F41" s="0">
-        <v>1008</v>
+      <c r="E10" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="F10" s="0">
+        <v>3388</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="C11" s="0" t="s">
+        <v>58</v>
+      </c>
+      <c r="D11" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="E11" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="F11" s="0">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="C12" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="D12" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="E12" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" s="0">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="B13" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="C13" s="0" t="s">
+        <v>60</v>
+      </c>
+      <c r="D13" s="0" t="s">
+        <v>88</v>
+      </c>
+      <c r="E13" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="F13" s="0">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="B14" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="C14" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="D14" s="0" t="s">
+        <v>89</v>
+      </c>
+      <c r="E14" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="F14" s="0">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="B15" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="C15" s="0" t="s">
+        <v>62</v>
+      </c>
+      <c r="D15" s="0" t="s">
+        <v>90</v>
+      </c>
+      <c r="E15" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="F15" s="0">
+        <v>15835</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="B16" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="C16" s="0" t="s">
+        <v>63</v>
+      </c>
+      <c r="D16" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="E16" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="F16" s="0">
+        <v>6480</v>
       </c>
     </row>
   </sheetData>

</xml_diff>